<commit_message>
working on what makes really functional categories
</commit_message>
<xml_diff>
--- a/data_Ref/bacteria_corrosion_summary.xlsx
+++ b/data_Ref/bacteria_corrosion_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -1061,10 +1061,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>872</t>
-        </is>
+      <c r="A31" s="1" t="n">
+        <v>872</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1083,6 +1081,451 @@
       </c>
       <c r="E31" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Actinomyces</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Actinomyces[Organism] AND corrosion[Title]: 7 hits; Actinomyces[Organism] AND (metal reduction OR iron reduction): 26 hits; Actinomyces[Organism] AND corrosion: 15 hits; Actinomyces[Organism] AND biocorrosion: 1 hits; Actinomyces[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 159 hits; Actinomyces[Organism] AND 'material deterioration': 1 hits; Actinomyces[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 11 hits; Actinomyces[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 17 hits; Actinomyces[Organism] AND AND biofilm AND (corrosion OR MIC): 45 hits</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Anaerococcus</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Anaerococcus[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 7 hits</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Aquabacter</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Aquabacterium</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Aquabacterium[Organism] AND corrosion[Title]: 1 hits; Aquabacterium[Organism] AND (metal reduction OR iron reduction): 8 hits; Aquabacterium[Organism] AND corrosion: 2 hits; Aquabacterium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 1 hits; Aquabacterium[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits; Aquabacterium[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Atopobium</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Atopobium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 9 hits; Atopobium[Organism] AND 'material deterioration': 1 hits; Atopobium[Organism] AND AND biofilm AND (corrosion OR MIC): 2 hits</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium[Organism] AND (metal reduction OR iron reduction): 4 hits; Cellulosimicrobium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 2 hits</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>214</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Clostridium</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Metal Reduction; Sulfate Reduction</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Clostridium[Organism] AND corrosion[Title]: 7 hits; Clostridium[Organism] AND biocorrosion[Title]: 1 hits; Clostridium[Organism] AND (metal reduction OR iron reduction): 601 hits; Clostridium[Organism] AND corrosion: 73 hits; Clostridium[Organism] AND biocorrosion: 4 hits; Clostridium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 700 hits; Clostridium[Organism] AND 'material deterioration': 16 hits; Clostridium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 26 hits; Clostridium[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 31 hits; Clostridium[Organism] AND AND biofilm AND (corrosion OR MIC): 29 hits; Clostridium[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 10 hits; Clostridium[Organism] AND (hydrogen sulfide OR H2S) AND (corrosion OR 'metal deterioration')Clostridium[Organism] AND ('sulfate reducing bacteria'[Title/Abstract] AND corrosion): 3 hits</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>225</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Colwellia</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Colwellia[Organism] AND corrosion[Title]: 20 hits; Colwellia[Organism] AND biocorrosion[Title]: 1 hits; Colwellia[Organism] AND 'microbiologically influenced corrosion'[Title]: 2 hits; Colwellia[Organism] AND (metal reduction OR iron reduction): 621 hits; Colwellia[Organism] AND corrosion: 48 hits; Colwellia[Organism] AND biocorrosion: 9 hits; Colwellia[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 47 hits; Colwellia[Organism] AND 'material deterioration': 3 hits; Colwellia[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 38 hits; Colwellia[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 6 hits; Colwellia[Organism] AND AND biofilm AND (corrosion OR MIC): 33 hits; Colwellia[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 20 hits; Colwellia[Organism] AND ('metal reducing bacteria'[Title/Abstract] AND corrosion): 1 hits</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>229</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Corynebacterium</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Corynebacterium[Organism] AND (metal reduction OR iron reduction): 67 hits; Corynebacterium[Organism] AND corrosion: 18 hits; Corynebacterium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 204 hits; Corynebacterium[Organism] AND 'material deterioration': 3 hits; Corynebacterium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 4 hits; Corynebacterium[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 14 hits; Corynebacterium[Organism] AND AND biofilm AND (corrosion OR MIC): 14 hits</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>334</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Gelria</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Gelria[Organism] AND (metal reduction OR iron reduction): 1 hits</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>342</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Georgfuchsia</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Georgfuchsia[Organism] AND (metal reduction OR iron reduction): 3 hits</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>351</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Haemophilus</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Haemophilus[Organism] AND (metal reduction OR iron reduction): 30 hits; Haemophilus[Organism] AND corrosion: 6 hits; Haemophilus[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 1520 hits; Haemophilus[Organism] AND 'material deterioration': 2 hits; Haemophilus[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 1 hits; Haemophilus[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 46 hits; Haemophilus[Organism] AND AND biofilm AND (corrosion OR MIC): 28 hits</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1633</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>426</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Lyngbya</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Lyngbya[Organism] AND (metal reduction OR iron reduction): 5 hits; Lyngbya[Organism] AND corrosion: 1 hits; Lyngbya[Organism] AND biocorrosion: 2 hits; Lyngbya[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 3 hits; Lyngbya[Organism] AND 'material deterioration': 1 hits; Lyngbya[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>471</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Mycoplana</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>480</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Nitratireductor</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Nitratireductor[Organism] AND (metal reduction OR iron reduction): 2 hits</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>494</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Oceaniovalibus</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Peptoclostridium</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>549</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Phenylobacterium</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Phenylobacterium[Organism] AND (metal reduction OR iron reduction): 2 hits; Phenylobacterium[Organism] AND corrosion: 1 hits</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>565</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Porphyromonas</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Porphyromonas[Organism] AND corrosion[Title]: 5 hits; Porphyromonas[Organism] AND biocorrosion[Title]: 1 hits; Porphyromonas[Organism] AND (metal reduction OR iron reduction): 74 hits; Porphyromonas[Organism] AND corrosion: 18 hits; Porphyromonas[Organism] AND biocorrosion: 3 hits; Porphyromonas[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 340 hits; Porphyromonas[Organism] AND 'material deterioration': 7 hits; Porphyromonas[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 17 hits; Porphyromonas[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 13 hits; Porphyromonas[Organism] AND AND biofilm AND (corrosion OR MIC): 113 hits</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>584</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas[Organism] AND corrosion[Title]: 4 hits; Pseudoalteromonas[Organism] AND 'microbiologically influenced corrosion'[Title]: 1 hits; Pseudoalteromonas[Organism] AND (metal reduction OR iron reduction): 16 hits; Pseudoalteromonas[Organism] AND corrosion: 14 hits; Pseudoalteromonas[Organism] AND biocorrosion: 3 hits; Pseudoalteromonas[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 17 hits; Pseudoalteromonas[Organism] AND 'material deterioration': 2 hits; Pseudoalteromonas[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 9 hits; Pseudoalteromonas[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 3 hits; Pseudoalteromonas[Organism] AND AND biofilm AND (corrosion OR MIC): 9 hits; Pseudoalteromonas[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Rhodanobacter</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Rhodanobacter[Organism] AND (metal reduction OR iron reduction): 18 hits; Rhodanobacter[Organism] AND corrosion: 1 hits; Rhodanobacter[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1096,7 +1539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -1622,10 +2065,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>872</t>
-        </is>
+      <c r="A31" s="1" t="n">
+        <v>872</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1642,6 +2083,372 @@
           <t>A two-chamber MFC system was operated continuously for more than 500 days to evaluate effects of biofilm and chemical scale formation on the cathode electrode on power generation. A stable power density of 0.57 W/m(2) was attained after 200 days operation. However, the power density decreased drastically to 0.2 W/m(2) after the cathodic biofilm and chemical scale were removed. As the cathodic biofilm and chemical scale partially accumulated on the cathode, the power density gradually recovered with time. Microbial community structure of the cathodic biofilm was analyzed based on 16S rRNA clone libraries. The clones closely related to Xanthomonadaceae bacterium and Xanthomonas sp. in the Gammaproteobacteria subdivision were most frequently retrieved from the cathodic biofilm. Results of the SEM-EDX analysis revealed that the cation species (Na(+) and Ca(2+)) were main constituents of chemical scale, indicating that these cations diffused from the anode chamber through the Nafion membrane. However, an excess accumulation of the biofilm and chemical scale on the cathode exhibited adverse effects on the power generation due to a decrease in the active cathode surface area and an increase in diffusion resistance for oxygen. Thus, it is important to properly control the formation of chemical scale and biofilm on the cathode during long-term operation.</t>
         </is>
       </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Actinomyces</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Sunil, M., Kurangi, B., Dodamani, S., Khalil, M. &amp; Chopra, A. (2025). Antimicrobial, antibiofilm, cytotoxicity, and substantivity of aged garlic extract against oral bacteria: an in-vitro study.. BMC complementary medicine and therapies, 25(1), 266.</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Garlic (Allium sativum L.) is a powerful antimicrobial, antioxidant, and anti-inflammatory agent. Aged garlic has more antioxidant and antimicrobial properties compared to fresh garlic. Garlic has been used for the treatment of many oral and periodontal diseases. However, the efficacy of aged garlic extract (AGE) against periodontal pathogens has never been explored. Hence, this in vitro study aims to assess the antimicrobial, antibiofilm, substantivity, and cytotoxic properties of AGE against key periodontal pathogens and oral tissues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Anaerococcus</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Akgül, Ö., Söyletir, G. &amp; Ülger Toprak, N. (2020). [Antimicrobial Susceptibility of Pathogenic Gram-positive Anaerobic Cocci: Data of a University Hospital in Turkey].. Mikrobiyoloji bulteni, 54(3), 404-417.</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Gram-positive anaerobic cocci (GPAC), a large group of anaerobic bacteria, are the members of the normal microbiota that colonizes the skin and mucosal surfaces of the human body. However, in case of a wound or when the host becomes immunocompromised, GPAC can cause invasive and most frequently mixed infections. GPAC are the second most frequently isolated bacteria in anaerobic infections. Although the studies are limited, GPAC have been reported to develop resistance to antimicrobial drugs. The resistance of the pathogens to the antimicrobials and improper therapy can cause poor clinical outcomes. Therefore, monitoring of the resistance trends of regional clinically important anaerobic bacteria periodically is recommended. In our study, we aimed to determine the antimicrobial susceptibility profiles of clinically important GPAC. A total of 100 non-duplicated pathogenic GPAC isolates were collected from Marmara University Hospital between 2013 and 2015. The isolates were identified by using conventional methods, "matrix-assisted laser desorption ionization-time of flight mass spectrometry system (MALDI-TOF MS)" (VITEK MS; v3.0, bioMerieux, France) and 16S rRNA gene sequencing. Antimicrobial susceptibility test was carried out by the agar dilution method according to the Clinical and Laboratory Standards Institute (CLSI) guidelines. The following antimicrobials were tested: penicillin, amoxicillin/ clavulanic acid (AMC), cefoxitin, meropenem, clindamycin, erythromycin, tetracycline, tigecycline, chloramphenicol, moxifloxacin and metronidazole. The minimum inhibitory concentration (MIC) results were interpreted according to the breakpoints described by the European Committee on Antimicrobial Susceptibility Testing (EUCAST). Breakpoints recommended by CLSI for cefoxitin, tetracycline and moxifloxacin, and breakpoint recommended by Food and Drug Administration (FDA) for tigecycline were used since there were no EUCAST breakpoints for these antimicrobials. MIC50 and MIC90 values were determined for erythromycin since the breakpoint was not described by EUCAST, CLSI or FDA guidelines. The identification results showed that the strains (n= 100) consisted of five different GPAC genus; Parvomonas (40%), Finegoldia (34%), Peptoniphilus (14%), Peptostreptococcus (10%) and Anaerococcus (1%). All of the organisms were susceptible to meropenem, tigecycline and metronidazole. The isolates were highly susceptible to penicillin, AMC, cefoxitin, and chloramphenicol, since the resistance rates against these antimicrobials were 5% or less. The resistance rates against clindamycin, tetracycline and moxifloxacin were 14%, 31% and 24%, respectively. In total, 11% of the isolates were multidrug resistant. Metronidazole and tigecycline displayed high in vitro activity against GPAC and both are appropriate antimicrobials for the selection of empiric therapy. The effectiveness of meropenem was also found high, but it was observed that this antimicrobial would be more appropriate to use in the treatment of severe mixed infections accompanied by other microorganisms with the resistance potential. Detection of penicillin and AMC resistant isolates, which are frequently used in the treatment of GPAC infection, requires periodic monitoring of the antimicrobial susceptibility patterns of GPAC. The high rates of resistance against clindamycin, tetracycline and moksifloxacin indicated that these antimicrobials should not be used for empirical treatment of infections without prior antimicrobial susceptibility testing. This study is one of the largest susceptibility studies specifically carried out on GPAC to date in Turkey. We believe that our results will provide good surveillance data both for our hospital and our country.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Aquabacter</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Aquabacterium</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Jin, J., Wu, G. &amp; Guan, Y. (2015). Effect of bacterial communities on the formation of cast iron corrosion tubercles in reclaimed water.. Water research, 71, 207-18.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>To understand the role bacterial communities play in corrosion scale development, the morphological and physicochemical characteristics of corrosion scales in raw and disinfected reclaimed water were systematically investigated. Corrosion tubercles were found in raw reclaimed water while thin corrosion layers formed in disinfected reclaimed water. The corrosion tubercles, composed mainly of α-FeOOH, γ-FeOOH, and CaCO3, consisted of an top surface; a shell containing more magnetite than other layers; a core in association with stalks produced by bacteria; and a corroded layer. The thin corrosion layers also had layered structures. These had a smooth top, a dense middle, and a corroded layer. They mostly consisted of the same main components as the tubercles in raw reclaimed water, but with different proportions. The profiles of the dissolved oxygen (DO) concentration, redox potential, and pH in the tubercles were different to those in the corrosion layers, which demonstrated that these parameters changed with a shift in the microbial processes in the tubercles. The bacterial communities in the tubercles were found to be dominated by Proteobacteria (56.7%), Bacteroidetes (10.0%), and Nitrospira (6.9%). The abundance of sequences affiliated to iron-reducing bacteria (IRB, mainly Geothrix) and iron-oxidizing bacteria (mainly Aquabacterium) was relatively high. The layered characteristics of the corrosion layers was due to the blocking of DO transfer by the development of the scales themselves. Bacterial communities could at least promote the layering process and formation of corrosion tubercles. Possible mechanisms might include: (1) bacterial communities mediated the pH and redox potential in the tubercles (which helped to form shell-like and core layers), (2) the metabolism of IRB and magnetic bacteria (Magnetospirillum) might contribute to the presence of Fe3O4 in the shell-like layer, while IRB contributed to green rust in the core layer, and (3) the diversity of the bacterial community resulted in the complex composition of the core layer, and gas producing bacteria (sulfate-reducing bacteria and methanogenic bacteria) played a role in the formation of the porous core layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Atopobium</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Rosca, A., Castro, J., Sousa, L., França, A., Vaneechoutte, M. &amp; Cerca, N. (2022). In vitro interactions within a biofilm containing three species found in bacterial vaginosis (BV) support the higher antimicrobial tolerance associated with BV recurrence.. The Journal of antimicrobial chemotherapy, 77(8), 2183-2190.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Bacterial vaginosis (BV), the most common cause of vaginal discharge, is characterized by the presence of a polymicrobial biofilm on the vaginal epithelium, formed primarily by Gardnerella spp., but also other anaerobic species. Interactions between bacteria in multi-species biofilms are likely to contribute to increased virulence and to enhanced antimicrobial tolerance observed in vivo. However, functional studies addressing this question are lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Bharagava, R. &amp; Mishra, S. (2018). Hexavalent chromium reduction potential of Cellulosimicrobium sp. isolated from common effluent treatment plant of tannery industries.. Ecotoxicology and environmental safety, 147, 102-109.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Present study deals with the isolation and characterization of a bacterium capable for the effective reduction of Cr(VI) from tannery wastewater. Based on the 16S rRNA gene sequence analysis, this bacterium was identified as Cellulosimicrobium sp. (KX710177). During the Cr(VI) reduction experiment performed at 50, 100, 200,and 300mg/L of Cr(VI) concentrations, the bacterium showed 99.33% and 96.98% reduction at 50 and 100mg/L at 24 and 96h, respectively. However, at 200 and 300mg/L concentration of Cr(VI), only 84.62% and 62.28% reduction was achieved after 96h, respectively. The SEM analysis revealed that bacterial cells exposed to Cr(VI) showed increased cell size in comparison to unexposed cells, which might be due to either the precipitation or adsorption of reduced Cr(III) on bacterial cells. Further, the Energy Dispersive X-ray (EDX) analysis showed some chromium peaks for cells exposed to Cr(VI), which might be either due to the presence of precipitated reduced Cr(III) on cells or complexation of Cr(III) with cell surface molecules. The bacterium also showed resistance and sensitivity against the tested antibiotics with a wide range of MIC values ranging from 250 to 800mg/L for different heavy metals. Thus, this multi-drug and multi-metal resistant bacterium can be used as a potential agent for the effective bioremediation of metal contaminated sites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>214</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Clostridium</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Ramos Monroy, O., Ruiz Ordaz, N., Hernández Gayosso, M., Juárez Ramírez, C. &amp; Galíndez Mayer, J. (2019). The corrosion process caused by the activity of the anaerobic sporulated bacterium Clostridium celerecrescens on API XL 52 steel.. Environmental science and pollution research international, 26(29), 29991-30002.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>The microbial corrosion of oil and gas pipes is one of the problems occurring in the oil industry. Various mechanisms explaining microbial corrosion have been demonstrated. Commonly, biocorrosion is attributed to sulfate-reducing bacteria. Also, it has recently been reported that microbial species can connect their electron transport system to metal electrodes. In this research, two spore-forming bacteria isolated in different years from a gas pipeline were identified by biochemical techniques and by 16S rDNA amplification, sequencing, and comparison with the NCBI database. Isolates were also compared between them using molecular techniques as the restriction patterns, unique for 16S rDNA (ARDRA), and the profile of the amplified bit from the genomic DNA, using an unspecific primer (RAPD). The results obtained showed that both isolates corresponded to Clostridium celerecrescens with a 99% similarity according to the sequence reported on the NCBI database. Also, the ARDRA and RAPD electrophoretic profiles of both strains were identical, and no plasmids were found in the strains. Thus, it can be settled that this bacterium is persistent in the environment prevailing in gas pipelines. Also, it was demonstrated that the bacterial secretion of organic acids contributes to the pitting and general biocorrosion of API XL 52 steel. The rates of corrosion obtained, approximately after 40 days, were correlated with the presence and metabolic activity of C. celerecrescens on the metallic surfaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>225</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Colwellia</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Zeng, Z., He, D., Zhao, Z., He, T., Li, Q. &amp; Wang, Y. (2025). A point mutation in a &lt;i&gt;wspF-&lt;/i&gt;like gene in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; enhances the anticorrosion activity.. Applied and environmental microbiology, 91(2), e0215424.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>The protection of steel based on microbial biomineralization has emerged as a novel and eco-friendly strategy for corrosion control. However, the molecular basis of the biomineralization process in mineralization bacteria remains largely unexplored. We previously reported that &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; EPS+ strain provides protection against steel corrosion by forming a hybrid biomineralization film. In this study, we identified that a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; (&lt;i&gt;wspF-&lt;/i&gt;like) gene, responsible for encoding a chemotaxis protein that regulates swimming motility and polysaccharide production, is linked to the observed anticorrosion activity in EPS+ strain. The engineered point mutation mutant strain, designated Δ&lt;i&gt;08765(707A&lt;/i&gt;), exhibited similar phenotypes to the EPS+ strain, including colony morphology and cellulose production. Importantly, we demonstrated that moderate swimming motility in Δ&lt;i&gt;08765(707A&lt;/i&gt;) plays a pivotal role in the development of a protective mineralization film on the steel surface. Additionally, we found that Δ&lt;i&gt;08765(707A&lt;/i&gt;) enhances biofilm formation by rapidly forming small aggregates in the initial stage of biofilm growth. This process facilitated the assembly of more compact and larger mineralization products, effectively inhibiting steel corrosion. In addition, Δ&lt;i&gt;08765(707A&lt;/i&gt;) formed a uniform mineralization film that completely covered the steel surface, preventing the formation of sheet-like steel corrosion products. Therefore, this study demonstrates that an engineering strain carrying a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; gene can significantly enhance the anticorrosion activity. This enhancement is accomplished through the formation of small bacteria-induced aggregates, followed by the development of larger mineralization products and the creation of a uniform organic-inorganic hybrid film.&lt;b&gt;IMPORTANCE&lt;/b&gt;In this study, we revealed that moderate swimming motility significantly influences the anticorrosion activity of marine &lt;i&gt;Pseudoalteromonas&lt;/i&gt;. Furthermore, our study demonstrated that overproduction of cellulose facilitates cell aggregation rapidly during the initial stages of biofilm formation, thereby promoting the development of larger mineralization products and the formation of a uniform organic-inorganic hybrid film on the steel surface. Our findings provide new insights into the biomineralization mechanisms in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt;, potentially catalyzing the advancement of an eco-friendly microbial-driven approach to marine corrosion prevention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>229</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Corynebacterium</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Aimo-Koivisto, E., Punakallio, L., Järvinen, R., Junnila, J., Grönthal, T. &amp; Rantala, M. (2024). A pilot study of antimicrobial effects and ototoxicity of a Norway spruce (Picea abies) resin-based canine otic rinse product.. Veterinary dermatology, 35(3), 325-336.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Norway spruce (Picea abies) resin-based products are used in human medicine. A resin-based otic rinse also could be useful in supportive care of canine otitis externa (COE), yet information on its antimicrobial effect against canine pathogens or ototoxicity is lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>334</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Gelria</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>342</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Georgfuchsia</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Atashgahi, S., et al. (2021). Proteogenomic analysis of Georgfuchsia toluolica revealed unexpected concurrent aerobic and anaerobic toluene degradation.. Environmental microbiology reports, 13(6), 841-851.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Denitrifying Betaproteobacteria play a key role in the anaerobic degradation of monoaromatic hydrocarbons. We performed a multi-omics study to better understand the metabolism of the representative organism Georgfuchsia toluolica strain G5G6 known as a strict anaerobe coupling toluene oxidation with dissimilatory nitrate and Fe(III) reduction. Despite the genomic potential for degradation of different carbon sources, we did not find sugar or organic acid transporters, in line with the inability of strain G5G6 to use these substrates. Using a proteomics analysis, we detected proteins of fumarate-dependent toluene activation, membrane-bound nitrate reductase, and key components of the metal-reducing (Mtr) pathway under both nitrate- and Fe(III)-reducing conditions. High abundance of the multiheme cytochrome MtrC implied that a porin-cytochrome complex was used for respiratory Fe(III) reduction. Remarkably, strain G5G6 contains a full set of genes for aerobic toluene degradation, and we detected enzymes of aerobic toluene degradation under both nitrate- and Fe(III)-reducing conditions. We further detected an ATP-dependent benzoyl-CoA reductase, reactive oxygen species detoxification proteins, and cytochrome c oxidase indicating a facultative anaerobic lifestyle of strain G5G6. Correspondingly, we found diffusion through the septa a substantial source of oxygen in the cultures enabling concurrent aerobic and anaerobic toluene degradation by strain G5G6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>351</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Haemophilus</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Xiao, J., Su, L., Huang, S., Zhou, M. &amp; Chen, Z. (2025). Integrated transcriptomics and metabolomics study on the biofilm formation of Haemophilus influenzae by the stimulation of amoxicillin-clavulanate at subinhibitory concentration.. Microbial pathogenesis, 205, 107650.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Exposure to subinhibitory concentrations of β-lactam antibiotics has been shown to induce the biofilm formation of microorganisms, but the underlying mechanisms remain poorly understood. This study aims to explore the effect of different concentrations of amoxicillin-clavulanate, the most commonly used antibiotic in pediatrics, on the biofilm formation of Haemophilus influenza (H. influenzae) in vitro and to explore the underlying mechanisms. The effect of amoxicillin-clavulanate on the in vitro biofilm formation was assessed by crystal violet assay, colony counts, MTT colorimetric method, scanning electron microscopy, and confocal laser scanning microscopy. Integrated transcriptomics and metabolomics analyses were performed to identify key genes and metabolites. Our findings revealed that 1/2 MIC of amoxicillin-clavulanate significantly enhanced H. influenzae ATCC 49247 biofilm formation in vitro, while simultaneously reducing culturable bacterial counts and metabolic activity of biofilm-embedded bacteria. When exposed to 1/2 MIC of amoxicillin-clavulanate, the biofilm ultrastructure was altered, with an increase in biofilm structure, a decrease in bacteria embedded within the biofilms with abnormal bacterial morphology. Transcriptomics identified 118 differentially expressed genes (DEGs), comprising 62 upregulated and 56 downregulated genes. Metabolomics identified 21 differentially expressed metabolites (DEMs), with 13 upregulated and 8 downregulated. Integrated transcriptomics and metabolomics implicated amino sugar and nucleotide sugar metabolism as a key regulatory pathway. This study has provided novel insights into the relationship between a commonly prescribed pediatric antibiotic and H. influenzae biofilm formation, elucidating the underlying mechanisms, emphasizing the critical importance of judicious antibiotic use and clinical consideration of subinhibitory antibiotic effects, particularly in pediatric populations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>426</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Lyngbya</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Parvin, N., Mandal, S. &amp; Rath, J. (2024). Microbiome of seventh-century old Parsurameswara stone monument of India and role of desiccation-tolerant cyanobacterium &lt;i&gt;Lyngbya corticicola&lt;/i&gt; on its biodeterioration.. Biofouling, 40(1), 40-53.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>The Parsurameswara stone monument, built in the seventh century, is one of the oldest stone monuments in Odisha, India. Metagenomic analysis of the biological crust samples collected from the stone monument revealed 17 phyla in the microbiome, with Proteobacteria being the most dominant phylum, followed by cyanobacteria. Eight cyanobacteria were isolated. &lt;i&gt;Lyngbya corticicola&lt;/i&gt; was the dominant cyanobacterium in all crust samples and could tolerate six months of desiccation &lt;i&gt;in vitro&lt;/i&gt;. With six months of desiccation, chlorophyll-&lt;i&gt;a&lt;/i&gt; decreased; however, carotenoid and cellular carbohydrate contents of this organism increased in the desiccated state. Resistance to desiccation, high carotenoid content, and effective trehalose biosynthesis in this cyanobacterium provide a distinct advantage over other microbiomes. Comparative metabolic profiles of the biological crust and &lt;i&gt;L. corticicola&lt;/i&gt; show strongly corrosive organic acids such as dichloroacetic acid, which might be responsible for the biocorrosion of stone monuments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>471</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Mycoplana</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>480</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Nitratireductor</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>494</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Oceaniovalibus</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Peptoclostridium</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>549</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Phenylobacterium</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Kalwasińska, A., Felföldi, T., Szabó, A., Deja-Sikora, E., Kosobucki, P. &amp; Walczak, M. (2017). Microbial communities associated with the anthropogenic, highly alkaline environment of a saline soda lime, Poland.. Antonie van Leeuwenhoek, 110(7), 945-962.</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Soda lime is a by-product of the Solvay soda process for the production of sodium carbonate from limestone and sodium chloride. Due to a high salt concentration and alkaline pH, the lime is considered as a potential habitat of haloalkaliphilic and haloalkalitolerant microbial communities. This artificial and unique environment is nutrient-poor and devoid of vegetation, due in part to semi-arid, saline and alkaline conditions. Samples taken from the surface layer of the lime and from the depth of 2 m (both having pH ~11 and EC&lt;sub&gt;e&lt;/sub&gt; up to 423 dS m&lt;sup&gt;-1&lt;/sup&gt;) were investigated using culture-based (culturing on alkaline medium) and culture-independent microbiological approaches (microscopic analyses and pyrosequencing). A surprisingly diverse bacterial community was discovered in this highly saline, alkaline and nutrient-poor environment, with the bacterial phyla Proteobacteria (representing 52.8% of the total bacterial community) and Firmicutes (16.6%) showing dominance. Compared to the surface layer, higher bacterial abundance and diversity values were detected in the deep zone, where more stable environmental conditions may occur. The surface layer was dominated by members of the genera Phenylobacterium, Chelativorans and Skermanella, while in the interior layer the genus Fictibacillus was dominant. The culturable aerobic, haloalkaliphilic bacteria strains isolated in this study belonged mostly to the genus Bacillus and were closely related to the species Bacillus pseudofirmus, B. cereus, B. plakortidis, B. thuringensis and B. pumilus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>565</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Porphyromonas</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Raza, F., Vaidyanathan, A., Kandasamy, R., Krishnaswami, V. &amp; Vijayaraghavalu, S. (2025). Synthesis of Surface-Charged IGF-1 Loaded PLGA Nanoparticles and Assess Dual Antimicrobial and Osteogenic Effects for Peri- Implant Bone Health: An In-Vitro Study.. The International journal of oral &amp; maxillofacial implants, 0(0), 1-31.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>To develop Insulin-like Growth Factor-1 (IGF-1)-loaded poly (lactic-co-glycolic acid)(PLGA) nanoparticles (NPs) with altered surface charges (cationic, anionic, and neutral) and evaluate their dual antimicrobial and osteogenic potential in vitro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>584</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Zeng, Z., He, D., Zhao, Z., He, T., Li, Q. &amp; Wang, Y. (2025). A point mutation in a &lt;i&gt;wspF-&lt;/i&gt;like gene in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; enhances the anticorrosion activity.. Applied and environmental microbiology, 91(2), e0215424.</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>The protection of steel based on microbial biomineralization has emerged as a novel and eco-friendly strategy for corrosion control. However, the molecular basis of the biomineralization process in mineralization bacteria remains largely unexplored. We previously reported that &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; EPS+ strain provides protection against steel corrosion by forming a hybrid biomineralization film. In this study, we identified that a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; (&lt;i&gt;wspF-&lt;/i&gt;like) gene, responsible for encoding a chemotaxis protein that regulates swimming motility and polysaccharide production, is linked to the observed anticorrosion activity in EPS+ strain. The engineered point mutation mutant strain, designated Δ&lt;i&gt;08765(707A&lt;/i&gt;), exhibited similar phenotypes to the EPS+ strain, including colony morphology and cellulose production. Importantly, we demonstrated that moderate swimming motility in Δ&lt;i&gt;08765(707A&lt;/i&gt;) plays a pivotal role in the development of a protective mineralization film on the steel surface. Additionally, we found that Δ&lt;i&gt;08765(707A&lt;/i&gt;) enhances biofilm formation by rapidly forming small aggregates in the initial stage of biofilm growth. This process facilitated the assembly of more compact and larger mineralization products, effectively inhibiting steel corrosion. In addition, Δ&lt;i&gt;08765(707A&lt;/i&gt;) formed a uniform mineralization film that completely covered the steel surface, preventing the formation of sheet-like steel corrosion products. Therefore, this study demonstrates that an engineering strain carrying a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; gene can significantly enhance the anticorrosion activity. This enhancement is accomplished through the formation of small bacteria-induced aggregates, followed by the development of larger mineralization products and the creation of a uniform organic-inorganic hybrid film.&lt;b&gt;IMPORTANCE&lt;/b&gt;In this study, we revealed that moderate swimming motility significantly influences the anticorrosion activity of marine &lt;i&gt;Pseudoalteromonas&lt;/i&gt;. Furthermore, our study demonstrated that overproduction of cellulose facilitates cell aggregation rapidly during the initial stages of biofilm formation, thereby promoting the development of larger mineralization products and the formation of a uniform organic-inorganic hybrid film on the steel surface. Our findings provide new insights into the biomineralization mechanisms in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt;, potentially catalyzing the advancement of an eco-friendly microbial-driven approach to marine corrosion prevention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Rhodanobacter</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
updating packages for warnings on notebook4
</commit_message>
<xml_diff>
--- a/data_Ref/bacteria_corrosion_summary.xlsx
+++ b/data_Ref/bacteria_corrosion_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -1504,10 +1504,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>605</t>
-        </is>
+      <c r="A52" s="1" t="n">
+        <v>605</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1526,6 +1524,634 @@
       </c>
       <c r="E52" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Actinomyces</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Actinomyces[Organism] AND corrosion[Title]: 7 hits; Actinomyces[Organism] AND (metal reduction OR iron reduction): 26 hits; Actinomyces[Organism] AND corrosion: 15 hits; Actinomyces[Organism] AND biocorrosion: 1 hits; Actinomyces[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 159 hits; Actinomyces[Organism] AND 'material deterioration': 1 hits; Actinomyces[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 11 hits; Actinomyces[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 17 hits; Actinomyces[Organism] AND AND biofilm AND (corrosion OR MIC): 45 hits</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Anaerococcus</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Anaerococcus[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 7 hits</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Aquabacter</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Aquabacterium</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Aquabacterium[Organism] AND corrosion[Title]: 1 hits; Aquabacterium[Organism] AND (metal reduction OR iron reduction): 8 hits; Aquabacterium[Organism] AND corrosion: 2 hits; Aquabacterium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 1 hits; Aquabacterium[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits; Aquabacterium[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Atopobium</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Atopobium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 9 hits; Atopobium[Organism] AND 'material deterioration': 1 hits; Atopobium[Organism] AND AND biofilm AND (corrosion OR MIC): 2 hits</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium[Organism] AND (metal reduction OR iron reduction): 4 hits; Cellulosimicrobium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 2 hits</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>214</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Clostridium</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Metal Reduction; Sulfate Reduction</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Clostridium[Organism] AND corrosion[Title]: 7 hits; Clostridium[Organism] AND biocorrosion[Title]: 1 hits; Clostridium[Organism] AND (metal reduction OR iron reduction): 602 hits; Clostridium[Organism] AND corrosion: 73 hits; Clostridium[Organism] AND biocorrosion: 4 hits; Clostridium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 700 hits; Clostridium[Organism] AND 'material deterioration': 16 hits; Clostridium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 26 hits; Clostridium[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 31 hits; Clostridium[Organism] AND AND biofilm AND (corrosion OR MIC): 29 hits; Clostridium[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 10 hits; Clostridium[Organism] AND (hydrogen sulfide OR H2S) AND (corrosion OR 'metal deterioration')Clostridium[Organism] AND ('sulfate reducing bacteria'[Title/Abstract] AND corrosion): 3 hits</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>225</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Colwellia</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Colwellia[Organism] AND corrosion[Title]: 20 hits; Colwellia[Organism] AND biocorrosion[Title]: 1 hits; Colwellia[Organism] AND 'microbiologically influenced corrosion'[Title]: 2 hits; Colwellia[Organism] AND (metal reduction OR iron reduction): 621 hits; Colwellia[Organism] AND corrosion: 48 hits; Colwellia[Organism] AND biocorrosion: 9 hits; Colwellia[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 47 hits; Colwellia[Organism] AND 'material deterioration': 3 hits; Colwellia[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 38 hits; Colwellia[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 6 hits; Colwellia[Organism] AND AND biofilm AND (corrosion OR MIC): 33 hits; Colwellia[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 20 hits; Colwellia[Organism] AND ('metal reducing bacteria'[Title/Abstract] AND corrosion): 1 hits</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>229</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Corynebacterium</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Corynebacterium[Organism] AND (metal reduction OR iron reduction): 67 hits; Corynebacterium[Organism] AND corrosion: 18 hits; Corynebacterium[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 204 hits; Corynebacterium[Organism] AND 'material deterioration': 3 hits; Corynebacterium[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 4 hits; Corynebacterium[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 14 hits; Corynebacterium[Organism] AND AND biofilm AND (corrosion OR MIC): 14 hits</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>334</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gelria</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Gelria[Organism] AND (metal reduction OR iron reduction): 1 hits</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>342</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Georgfuchsia</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Georgfuchsia[Organism] AND (metal reduction OR iron reduction): 3 hits</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>351</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Haemophilus</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Haemophilus[Organism] AND (metal reduction OR iron reduction): 30 hits; Haemophilus[Organism] AND corrosion: 6 hits; Haemophilus[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 1520 hits; Haemophilus[Organism] AND 'material deterioration': 2 hits; Haemophilus[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 1 hits; Haemophilus[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 46 hits; Haemophilus[Organism] AND AND biofilm AND (corrosion OR MIC): 28 hits</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1633</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>426</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Lyngbya</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Lyngbya[Organism] AND (metal reduction OR iron reduction): 5 hits; Lyngbya[Organism] AND corrosion: 1 hits; Lyngbya[Organism] AND biocorrosion: 2 hits; Lyngbya[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 3 hits; Lyngbya[Organism] AND 'material deterioration': 1 hits; Lyngbya[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>471</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mycoplana</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>480</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Nitratireductor</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Nitratireductor[Organism] AND (metal reduction OR iron reduction): 2 hits</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>494</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Oceaniovalibus</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Peptoclostridium</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>549</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Phenylobacterium</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Phenylobacterium[Organism] AND (metal reduction OR iron reduction): 2 hits; Phenylobacterium[Organism] AND corrosion: 1 hits</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>565</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Porphyromonas</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Porphyromonas[Organism] AND corrosion[Title]: 5 hits; Porphyromonas[Organism] AND biocorrosion[Title]: 1 hits; Porphyromonas[Organism] AND (metal reduction OR iron reduction): 74 hits; Porphyromonas[Organism] AND corrosion: 18 hits; Porphyromonas[Organism] AND biocorrosion: 3 hits; Porphyromonas[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 340 hits; Porphyromonas[Organism] AND 'material deterioration': 7 hits; Porphyromonas[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 17 hits; Porphyromonas[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 13 hits; Porphyromonas[Organism] AND AND biofilm AND (corrosion OR MIC): 113 hits</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>584</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas[Organism] AND corrosion[Title]: 4 hits; Pseudoalteromonas[Organism] AND 'microbiologically influenced corrosion'[Title]: 1 hits; Pseudoalteromonas[Organism] AND (metal reduction OR iron reduction): 16 hits; Pseudoalteromonas[Organism] AND corrosion: 14 hits; Pseudoalteromonas[Organism] AND biocorrosion: 3 hits; Pseudoalteromonas[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 17 hits; Pseudoalteromonas[Organism] AND 'material deterioration': 2 hits; Pseudoalteromonas[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 9 hits; Pseudoalteromonas[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 3 hits; Pseudoalteromonas[Organism] AND AND biofilm AND (corrosion OR MIC): 9 hits; Pseudoalteromonas[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>605</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Rhodanobacter</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Rhodanobacter[Organism] AND (metal reduction OR iron reduction): 18 hits; Rhodanobacter[Organism] AND corrosion: 1 hits; Rhodanobacter[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>625</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roseococcus</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Roseococcus[Organism] AND (metal reduction OR iron reduction): 1 hits; Roseococcus[Organism] AND corrosion: 1 hits</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>636</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Ruminococcaceae_ucg-005</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>657</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Shinella</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Shinella[Organism] AND (metal reduction OR iron reduction): 4 hits; Shinella[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 1 hits; Shinella[Organism] AND 'material deterioration': 1 hits</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>678</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Sphingosinicella</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>712</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Tepidimonas</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>725</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Thermus</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Thermus[Organism] AND corrosion[Title]: 1 hits; Thermus[Organism] AND 'microbiologically influenced corrosion'[Title]: 1 hits; Thermus[Organism] AND (metal reduction OR iron reduction): 144 hits; Thermus[Organism] AND corrosion: 2 hits; Thermus[Organism] AND biocorrosion: 2 hits; Thermus[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 12 hits; Thermus[Organism] AND 'material deterioration': 1 hits; Thermus[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 2 hits; Thermus[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 2 hits; Thermus[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits; Thermus[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 1 hits</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>864</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Veillonella</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Veillonella[Organism] AND corrosion[Title]: 2 hits; Veillonella[Organism] AND (metal reduction OR iron reduction): 13 hits; Veillonella[Organism] AND corrosion: 6 hits; Veillonella[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 56 hits; Veillonella[Organism] AND 'material deterioration': 1 hits; Veillonella[Organism] AND ('metal deterioration' OR 'metallic corrosion'): 3 hits; Veillonella[Organism] AND (acid production) AND (corrosion OR 'metal deterioration' OR MIC): 2 hits; Veillonella[Organism] AND AND biofilm AND (corrosion OR MIC): 11 hits; Veillonella[Organism] AND (ochre formation OR iron oxide deposits OR rust formation): 2 hits</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>871</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Xanthobacter</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Xanthobacter[Organism] AND (metal reduction OR iron reduction): 11 hits; Xanthobacter[Organism] AND (MIC OR 'microbiologically influenced corrosion'): 1 hits; Xanthobacter[Organism] AND 'material deterioration': 1 hits; Xanthobacter[Organism] AND AND biofilm AND (corrosion OR MIC): 1 hits</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>872</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Xanthomonadaceae_bacterium_wwh73</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Metal Reduction</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Xanthomonadaceae_bacterium_wwh73[Organism] AND (metal reduction OR iron reduction): 1 hits</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1539,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -2437,10 +3063,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>605</t>
-        </is>
+      <c r="A52" s="1" t="n">
+        <v>605</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2449,6 +3073,528 @@
       </c>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Actinomyces</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Sunil, M., Kurangi, B., Dodamani, S., Khalil, M. &amp; Chopra, A. (2025). Antimicrobial, antibiofilm, cytotoxicity, and substantivity of aged garlic extract against oral bacteria: an in-vitro study.. BMC complementary medicine and therapies, 25(1), 266.</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Garlic (Allium sativum L.) is a powerful antimicrobial, antioxidant, and anti-inflammatory agent. Aged garlic has more antioxidant and antimicrobial properties compared to fresh garlic. Garlic has been used for the treatment of many oral and periodontal diseases. However, the efficacy of aged garlic extract (AGE) against periodontal pathogens has never been explored. Hence, this in vitro study aims to assess the antimicrobial, antibiofilm, substantivity, and cytotoxic properties of AGE against key periodontal pathogens and oral tissues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Anaerococcus</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Akgül, Ö., Söyletir, G. &amp; Ülger Toprak, N. (2020). [Antimicrobial Susceptibility of Pathogenic Gram-positive Anaerobic Cocci: Data of a University Hospital in Turkey].. Mikrobiyoloji bulteni, 54(3), 404-417.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Gram-positive anaerobic cocci (GPAC), a large group of anaerobic bacteria, are the members of the normal microbiota that colonizes the skin and mucosal surfaces of the human body. However, in case of a wound or when the host becomes immunocompromised, GPAC can cause invasive and most frequently mixed infections. GPAC are the second most frequently isolated bacteria in anaerobic infections. Although the studies are limited, GPAC have been reported to develop resistance to antimicrobial drugs. The resistance of the pathogens to the antimicrobials and improper therapy can cause poor clinical outcomes. Therefore, monitoring of the resistance trends of regional clinically important anaerobic bacteria periodically is recommended. In our study, we aimed to determine the antimicrobial susceptibility profiles of clinically important GPAC. A total of 100 non-duplicated pathogenic GPAC isolates were collected from Marmara University Hospital between 2013 and 2015. The isolates were identified by using conventional methods, "matrix-assisted laser desorption ionization-time of flight mass spectrometry system (MALDI-TOF MS)" (VITEK MS; v3.0, bioMerieux, France) and 16S rRNA gene sequencing. Antimicrobial susceptibility test was carried out by the agar dilution method according to the Clinical and Laboratory Standards Institute (CLSI) guidelines. The following antimicrobials were tested: penicillin, amoxicillin/ clavulanic acid (AMC), cefoxitin, meropenem, clindamycin, erythromycin, tetracycline, tigecycline, chloramphenicol, moxifloxacin and metronidazole. The minimum inhibitory concentration (MIC) results were interpreted according to the breakpoints described by the European Committee on Antimicrobial Susceptibility Testing (EUCAST). Breakpoints recommended by CLSI for cefoxitin, tetracycline and moxifloxacin, and breakpoint recommended by Food and Drug Administration (FDA) for tigecycline were used since there were no EUCAST breakpoints for these antimicrobials. MIC50 and MIC90 values were determined for erythromycin since the breakpoint was not described by EUCAST, CLSI or FDA guidelines. The identification results showed that the strains (n= 100) consisted of five different GPAC genus; Parvomonas (40%), Finegoldia (34%), Peptoniphilus (14%), Peptostreptococcus (10%) and Anaerococcus (1%). All of the organisms were susceptible to meropenem, tigecycline and metronidazole. The isolates were highly susceptible to penicillin, AMC, cefoxitin, and chloramphenicol, since the resistance rates against these antimicrobials were 5% or less. The resistance rates against clindamycin, tetracycline and moxifloxacin were 14%, 31% and 24%, respectively. In total, 11% of the isolates were multidrug resistant. Metronidazole and tigecycline displayed high in vitro activity against GPAC and both are appropriate antimicrobials for the selection of empiric therapy. The effectiveness of meropenem was also found high, but it was observed that this antimicrobial would be more appropriate to use in the treatment of severe mixed infections accompanied by other microorganisms with the resistance potential. Detection of penicillin and AMC resistant isolates, which are frequently used in the treatment of GPAC infection, requires periodic monitoring of the antimicrobial susceptibility patterns of GPAC. The high rates of resistance against clindamycin, tetracycline and moksifloxacin indicated that these antimicrobials should not be used for empirical treatment of infections without prior antimicrobial susceptibility testing. This study is one of the largest susceptibility studies specifically carried out on GPAC to date in Turkey. We believe that our results will provide good surveillance data both for our hospital and our country.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Aquabacter</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Aquabacterium</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Jin, J., Wu, G. &amp; Guan, Y. (2015). Effect of bacterial communities on the formation of cast iron corrosion tubercles in reclaimed water.. Water research, 71, 207-18.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>To understand the role bacterial communities play in corrosion scale development, the morphological and physicochemical characteristics of corrosion scales in raw and disinfected reclaimed water were systematically investigated. Corrosion tubercles were found in raw reclaimed water while thin corrosion layers formed in disinfected reclaimed water. The corrosion tubercles, composed mainly of α-FeOOH, γ-FeOOH, and CaCO3, consisted of an top surface; a shell containing more magnetite than other layers; a core in association with stalks produced by bacteria; and a corroded layer. The thin corrosion layers also had layered structures. These had a smooth top, a dense middle, and a corroded layer. They mostly consisted of the same main components as the tubercles in raw reclaimed water, but with different proportions. The profiles of the dissolved oxygen (DO) concentration, redox potential, and pH in the tubercles were different to those in the corrosion layers, which demonstrated that these parameters changed with a shift in the microbial processes in the tubercles. The bacterial communities in the tubercles were found to be dominated by Proteobacteria (56.7%), Bacteroidetes (10.0%), and Nitrospira (6.9%). The abundance of sequences affiliated to iron-reducing bacteria (IRB, mainly Geothrix) and iron-oxidizing bacteria (mainly Aquabacterium) was relatively high. The layered characteristics of the corrosion layers was due to the blocking of DO transfer by the development of the scales themselves. Bacterial communities could at least promote the layering process and formation of corrosion tubercles. Possible mechanisms might include: (1) bacterial communities mediated the pH and redox potential in the tubercles (which helped to form shell-like and core layers), (2) the metabolism of IRB and magnetic bacteria (Magnetospirillum) might contribute to the presence of Fe3O4 in the shell-like layer, while IRB contributed to green rust in the core layer, and (3) the diversity of the bacterial community resulted in the complex composition of the core layer, and gas producing bacteria (sulfate-reducing bacteria and methanogenic bacteria) played a role in the formation of the porous core layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Atopobium</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Rosca, A., Castro, J., Sousa, L., França, A., Vaneechoutte, M. &amp; Cerca, N. (2022). In vitro interactions within a biofilm containing three species found in bacterial vaginosis (BV) support the higher antimicrobial tolerance associated with BV recurrence.. The Journal of antimicrobial chemotherapy, 77(8), 2183-2190.</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Bacterial vaginosis (BV), the most common cause of vaginal discharge, is characterized by the presence of a polymicrobial biofilm on the vaginal epithelium, formed primarily by Gardnerella spp., but also other anaerobic species. Interactions between bacteria in multi-species biofilms are likely to contribute to increased virulence and to enhanced antimicrobial tolerance observed in vivo. However, functional studies addressing this question are lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>201</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Cellulosimicrobium</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Bharagava, R. &amp; Mishra, S. (2018). Hexavalent chromium reduction potential of Cellulosimicrobium sp. isolated from common effluent treatment plant of tannery industries.. Ecotoxicology and environmental safety, 147, 102-109.</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Present study deals with the isolation and characterization of a bacterium capable for the effective reduction of Cr(VI) from tannery wastewater. Based on the 16S rRNA gene sequence analysis, this bacterium was identified as Cellulosimicrobium sp. (KX710177). During the Cr(VI) reduction experiment performed at 50, 100, 200,and 300mg/L of Cr(VI) concentrations, the bacterium showed 99.33% and 96.98% reduction at 50 and 100mg/L at 24 and 96h, respectively. However, at 200 and 300mg/L concentration of Cr(VI), only 84.62% and 62.28% reduction was achieved after 96h, respectively. The SEM analysis revealed that bacterial cells exposed to Cr(VI) showed increased cell size in comparison to unexposed cells, which might be due to either the precipitation or adsorption of reduced Cr(III) on bacterial cells. Further, the Energy Dispersive X-ray (EDX) analysis showed some chromium peaks for cells exposed to Cr(VI), which might be either due to the presence of precipitated reduced Cr(III) on cells or complexation of Cr(III) with cell surface molecules. The bacterium also showed resistance and sensitivity against the tested antibiotics with a wide range of MIC values ranging from 250 to 800mg/L for different heavy metals. Thus, this multi-drug and multi-metal resistant bacterium can be used as a potential agent for the effective bioremediation of metal contaminated sites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>214</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Clostridium</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Ramos Monroy, O., Ruiz Ordaz, N., Hernández Gayosso, M., Juárez Ramírez, C. &amp; Galíndez Mayer, J. (2019). The corrosion process caused by the activity of the anaerobic sporulated bacterium Clostridium celerecrescens on API XL 52 steel.. Environmental science and pollution research international, 26(29), 29991-30002.</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>The microbial corrosion of oil and gas pipes is one of the problems occurring in the oil industry. Various mechanisms explaining microbial corrosion have been demonstrated. Commonly, biocorrosion is attributed to sulfate-reducing bacteria. Also, it has recently been reported that microbial species can connect their electron transport system to metal electrodes. In this research, two spore-forming bacteria isolated in different years from a gas pipeline were identified by biochemical techniques and by 16S rDNA amplification, sequencing, and comparison with the NCBI database. Isolates were also compared between them using molecular techniques as the restriction patterns, unique for 16S rDNA (ARDRA), and the profile of the amplified bit from the genomic DNA, using an unspecific primer (RAPD). The results obtained showed that both isolates corresponded to Clostridium celerecrescens with a 99% similarity according to the sequence reported on the NCBI database. Also, the ARDRA and RAPD electrophoretic profiles of both strains were identical, and no plasmids were found in the strains. Thus, it can be settled that this bacterium is persistent in the environment prevailing in gas pipelines. Also, it was demonstrated that the bacterial secretion of organic acids contributes to the pitting and general biocorrosion of API XL 52 steel. The rates of corrosion obtained, approximately after 40 days, were correlated with the presence and metabolic activity of C. celerecrescens on the metallic surfaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>225</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Colwellia</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Zeng, Z., He, D., Zhao, Z., He, T., Li, Q. &amp; Wang, Y. (2025). A point mutation in a &lt;i&gt;wspF-&lt;/i&gt;like gene in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; enhances the anticorrosion activity.. Applied and environmental microbiology, 91(2), e0215424.</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>The protection of steel based on microbial biomineralization has emerged as a novel and eco-friendly strategy for corrosion control. However, the molecular basis of the biomineralization process in mineralization bacteria remains largely unexplored. We previously reported that &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; EPS+ strain provides protection against steel corrosion by forming a hybrid biomineralization film. In this study, we identified that a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; (&lt;i&gt;wspF-&lt;/i&gt;like) gene, responsible for encoding a chemotaxis protein that regulates swimming motility and polysaccharide production, is linked to the observed anticorrosion activity in EPS+ strain. The engineered point mutation mutant strain, designated Δ&lt;i&gt;08765(707A&lt;/i&gt;), exhibited similar phenotypes to the EPS+ strain, including colony morphology and cellulose production. Importantly, we demonstrated that moderate swimming motility in Δ&lt;i&gt;08765(707A&lt;/i&gt;) plays a pivotal role in the development of a protective mineralization film on the steel surface. Additionally, we found that Δ&lt;i&gt;08765(707A&lt;/i&gt;) enhances biofilm formation by rapidly forming small aggregates in the initial stage of biofilm growth. This process facilitated the assembly of more compact and larger mineralization products, effectively inhibiting steel corrosion. In addition, Δ&lt;i&gt;08765(707A&lt;/i&gt;) formed a uniform mineralization film that completely covered the steel surface, preventing the formation of sheet-like steel corrosion products. Therefore, this study demonstrates that an engineering strain carrying a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; gene can significantly enhance the anticorrosion activity. This enhancement is accomplished through the formation of small bacteria-induced aggregates, followed by the development of larger mineralization products and the creation of a uniform organic-inorganic hybrid film.&lt;b&gt;IMPORTANCE&lt;/b&gt;In this study, we revealed that moderate swimming motility significantly influences the anticorrosion activity of marine &lt;i&gt;Pseudoalteromonas&lt;/i&gt;. Furthermore, our study demonstrated that overproduction of cellulose facilitates cell aggregation rapidly during the initial stages of biofilm formation, thereby promoting the development of larger mineralization products and the formation of a uniform organic-inorganic hybrid film on the steel surface. Our findings provide new insights into the biomineralization mechanisms in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt;, potentially catalyzing the advancement of an eco-friendly microbial-driven approach to marine corrosion prevention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>229</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Corynebacterium</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Aimo-Koivisto, E., Punakallio, L., Järvinen, R., Junnila, J., Grönthal, T. &amp; Rantala, M. (2024). A pilot study of antimicrobial effects and ototoxicity of a Norway spruce (Picea abies) resin-based canine otic rinse product.. Veterinary dermatology, 35(3), 325-336.</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Norway spruce (Picea abies) resin-based products are used in human medicine. A resin-based otic rinse also could be useful in supportive care of canine otitis externa (COE), yet information on its antimicrobial effect against canine pathogens or ototoxicity is lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>334</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gelria</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>342</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Georgfuchsia</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Atashgahi, S., et al. (2021). Proteogenomic analysis of Georgfuchsia toluolica revealed unexpected concurrent aerobic and anaerobic toluene degradation.. Environmental microbiology reports, 13(6), 841-851.</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Denitrifying Betaproteobacteria play a key role in the anaerobic degradation of monoaromatic hydrocarbons. We performed a multi-omics study to better understand the metabolism of the representative organism Georgfuchsia toluolica strain G5G6 known as a strict anaerobe coupling toluene oxidation with dissimilatory nitrate and Fe(III) reduction. Despite the genomic potential for degradation of different carbon sources, we did not find sugar or organic acid transporters, in line with the inability of strain G5G6 to use these substrates. Using a proteomics analysis, we detected proteins of fumarate-dependent toluene activation, membrane-bound nitrate reductase, and key components of the metal-reducing (Mtr) pathway under both nitrate- and Fe(III)-reducing conditions. High abundance of the multiheme cytochrome MtrC implied that a porin-cytochrome complex was used for respiratory Fe(III) reduction. Remarkably, strain G5G6 contains a full set of genes for aerobic toluene degradation, and we detected enzymes of aerobic toluene degradation under both nitrate- and Fe(III)-reducing conditions. We further detected an ATP-dependent benzoyl-CoA reductase, reactive oxygen species detoxification proteins, and cytochrome c oxidase indicating a facultative anaerobic lifestyle of strain G5G6. Correspondingly, we found diffusion through the septa a substantial source of oxygen in the cultures enabling concurrent aerobic and anaerobic toluene degradation by strain G5G6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>351</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Haemophilus</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Xiao, J., Su, L., Huang, S., Zhou, M. &amp; Chen, Z. (2025). Integrated transcriptomics and metabolomics study on the biofilm formation of Haemophilus influenzae by the stimulation of amoxicillin-clavulanate at subinhibitory concentration.. Microbial pathogenesis, 205, 107650.</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Exposure to subinhibitory concentrations of β-lactam antibiotics has been shown to induce the biofilm formation of microorganisms, but the underlying mechanisms remain poorly understood. This study aims to explore the effect of different concentrations of amoxicillin-clavulanate, the most commonly used antibiotic in pediatrics, on the biofilm formation of Haemophilus influenza (H. influenzae) in vitro and to explore the underlying mechanisms. The effect of amoxicillin-clavulanate on the in vitro biofilm formation was assessed by crystal violet assay, colony counts, MTT colorimetric method, scanning electron microscopy, and confocal laser scanning microscopy. Integrated transcriptomics and metabolomics analyses were performed to identify key genes and metabolites. Our findings revealed that 1/2 MIC of amoxicillin-clavulanate significantly enhanced H. influenzae ATCC 49247 biofilm formation in vitro, while simultaneously reducing culturable bacterial counts and metabolic activity of biofilm-embedded bacteria. When exposed to 1/2 MIC of amoxicillin-clavulanate, the biofilm ultrastructure was altered, with an increase in biofilm structure, a decrease in bacteria embedded within the biofilms with abnormal bacterial morphology. Transcriptomics identified 118 differentially expressed genes (DEGs), comprising 62 upregulated and 56 downregulated genes. Metabolomics identified 21 differentially expressed metabolites (DEMs), with 13 upregulated and 8 downregulated. Integrated transcriptomics and metabolomics implicated amino sugar and nucleotide sugar metabolism as a key regulatory pathway. This study has provided novel insights into the relationship between a commonly prescribed pediatric antibiotic and H. influenzae biofilm formation, elucidating the underlying mechanisms, emphasizing the critical importance of judicious antibiotic use and clinical consideration of subinhibitory antibiotic effects, particularly in pediatric populations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>426</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Lyngbya</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Parvin, N., Mandal, S. &amp; Rath, J. (2024). Microbiome of seventh-century old Parsurameswara stone monument of India and role of desiccation-tolerant cyanobacterium &lt;i&gt;Lyngbya corticicola&lt;/i&gt; on its biodeterioration.. Biofouling, 40(1), 40-53.</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>The Parsurameswara stone monument, built in the seventh century, is one of the oldest stone monuments in Odisha, India. Metagenomic analysis of the biological crust samples collected from the stone monument revealed 17 phyla in the microbiome, with Proteobacteria being the most dominant phylum, followed by cyanobacteria. Eight cyanobacteria were isolated. &lt;i&gt;Lyngbya corticicola&lt;/i&gt; was the dominant cyanobacterium in all crust samples and could tolerate six months of desiccation &lt;i&gt;in vitro&lt;/i&gt;. With six months of desiccation, chlorophyll-&lt;i&gt;a&lt;/i&gt; decreased; however, carotenoid and cellular carbohydrate contents of this organism increased in the desiccated state. Resistance to desiccation, high carotenoid content, and effective trehalose biosynthesis in this cyanobacterium provide a distinct advantage over other microbiomes. Comparative metabolic profiles of the biological crust and &lt;i&gt;L. corticicola&lt;/i&gt; show strongly corrosive organic acids such as dichloroacetic acid, which might be responsible for the biocorrosion of stone monuments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>471</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mycoplana</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>480</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Nitratireductor</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr"/>
+      <c r="D67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>494</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Oceaniovalibus</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>541</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Peptoclostridium</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>549</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Phenylobacterium</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Kalwasińska, A., Felföldi, T., Szabó, A., Deja-Sikora, E., Kosobucki, P. &amp; Walczak, M. (2017). Microbial communities associated with the anthropogenic, highly alkaline environment of a saline soda lime, Poland.. Antonie van Leeuwenhoek, 110(7), 945-962.</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Soda lime is a by-product of the Solvay soda process for the production of sodium carbonate from limestone and sodium chloride. Due to a high salt concentration and alkaline pH, the lime is considered as a potential habitat of haloalkaliphilic and haloalkalitolerant microbial communities. This artificial and unique environment is nutrient-poor and devoid of vegetation, due in part to semi-arid, saline and alkaline conditions. Samples taken from the surface layer of the lime and from the depth of 2 m (both having pH ~11 and EC&lt;sub&gt;e&lt;/sub&gt; up to 423 dS m&lt;sup&gt;-1&lt;/sup&gt;) were investigated using culture-based (culturing on alkaline medium) and culture-independent microbiological approaches (microscopic analyses and pyrosequencing). A surprisingly diverse bacterial community was discovered in this highly saline, alkaline and nutrient-poor environment, with the bacterial phyla Proteobacteria (representing 52.8% of the total bacterial community) and Firmicutes (16.6%) showing dominance. Compared to the surface layer, higher bacterial abundance and diversity values were detected in the deep zone, where more stable environmental conditions may occur. The surface layer was dominated by members of the genera Phenylobacterium, Chelativorans and Skermanella, while in the interior layer the genus Fictibacillus was dominant. The culturable aerobic, haloalkaliphilic bacteria strains isolated in this study belonged mostly to the genus Bacillus and were closely related to the species Bacillus pseudofirmus, B. cereus, B. plakortidis, B. thuringensis and B. pumilus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>565</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Porphyromonas</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Raza, F., Vaidyanathan, A., Kandasamy, R., Krishnaswami, V. &amp; Vijayaraghavalu, S. (2025). Synthesis of Surface-Charged IGF-1 Loaded PLGA Nanoparticles and Assess Dual Antimicrobial and Osteogenic Effects for Peri- Implant Bone Health: An In-Vitro Study.. The International journal of oral &amp; maxillofacial implants, 0(0), 1-31.</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>To develop Insulin-like Growth Factor-1 (IGF-1)-loaded poly (lactic-co-glycolic acid)(PLGA) nanoparticles (NPs) with altered surface charges (cationic, anionic, and neutral) and evaluate their dual antimicrobial and osteogenic potential in vitro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>584</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pseudoalteromonas</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Zeng, Z., He, D., Zhao, Z., He, T., Li, Q. &amp; Wang, Y. (2025). A point mutation in a &lt;i&gt;wspF-&lt;/i&gt;like gene in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; enhances the anticorrosion activity.. Applied and environmental microbiology, 91(2), e0215424.</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>The protection of steel based on microbial biomineralization has emerged as a novel and eco-friendly strategy for corrosion control. However, the molecular basis of the biomineralization process in mineralization bacteria remains largely unexplored. We previously reported that &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt; EPS+ strain provides protection against steel corrosion by forming a hybrid biomineralization film. In this study, we identified that a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; (&lt;i&gt;wspF-&lt;/i&gt;like) gene, responsible for encoding a chemotaxis protein that regulates swimming motility and polysaccharide production, is linked to the observed anticorrosion activity in EPS+ strain. The engineered point mutation mutant strain, designated Δ&lt;i&gt;08765(707A&lt;/i&gt;), exhibited similar phenotypes to the EPS+ strain, including colony morphology and cellulose production. Importantly, we demonstrated that moderate swimming motility in Δ&lt;i&gt;08765(707A&lt;/i&gt;) plays a pivotal role in the development of a protective mineralization film on the steel surface. Additionally, we found that Δ&lt;i&gt;08765(707A&lt;/i&gt;) enhances biofilm formation by rapidly forming small aggregates in the initial stage of biofilm growth. This process facilitated the assembly of more compact and larger mineralization products, effectively inhibiting steel corrosion. In addition, Δ&lt;i&gt;08765(707A&lt;/i&gt;) formed a uniform mineralization film that completely covered the steel surface, preventing the formation of sheet-like steel corrosion products. Therefore, this study demonstrates that an engineering strain carrying a point mutation in the &lt;i&gt;AT00_08765&lt;/i&gt; gene can significantly enhance the anticorrosion activity. This enhancement is accomplished through the formation of small bacteria-induced aggregates, followed by the development of larger mineralization products and the creation of a uniform organic-inorganic hybrid film.&lt;b&gt;IMPORTANCE&lt;/b&gt;In this study, we revealed that moderate swimming motility significantly influences the anticorrosion activity of marine &lt;i&gt;Pseudoalteromonas&lt;/i&gt;. Furthermore, our study demonstrated that overproduction of cellulose facilitates cell aggregation rapidly during the initial stages of biofilm formation, thereby promoting the development of larger mineralization products and the formation of a uniform organic-inorganic hybrid film on the steel surface. Our findings provide new insights into the biomineralization mechanisms in &lt;i&gt;Pseudoalteromonas lipolytica&lt;/i&gt;, potentially catalyzing the advancement of an eco-friendly microbial-driven approach to marine corrosion prevention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>605</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Rhodanobacter</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>625</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roseococcus</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Ruiz-Lopez, S., Foster, L., Boothman, C., Cole, N., Morris, K. &amp; Lloyd, J. (2020). Identification of a Stable Hydrogen-Driven Microbiome in a Highly Radioactive Storage Facility on the Sellafield Site.. Frontiers in microbiology, 11, 587556.</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>The use of nuclear power has been a significant part of the United Kingdom's energy portfolio with the Sellafield site being used for power production and more recently reprocessing and decommissioning of spent nuclear fuel activities. Before being reprocessed, spent nuclear fuel is stored in water ponds with significant levels of background radioactivity and in high alkalinity (to minimize fuel corrosion). Despite these challenging conditions, the presence of microbial communities has been detected. To gain further insight into the microbial communities present in extreme environments, an indoor, hyper-alkaline, oligotrophic, and radioactive spent fuel storage pond (INP) located on the Sellafield site was analyzed. Water samples were collected from sample points within the INP complex, and also the purge water feeding tank (FT) that supplies water to the pond, and were screened for the presence of the 16S and 18S rRNA genes to inform sequencing requirements over a period of 30 months. Only 16S rRNA genes were successfully amplified for sequencing, suggesting that the microbial communities in the INP were dominated by prokaryotes. Quantitative Polymerase Chain Reaction (qPCR) analysis targeting 16S rRNA genes suggested that bacterial cells in the order of 10&lt;sup&gt;4&lt;/sup&gt;-10&lt;sup&gt;6&lt;/sup&gt; mL&lt;sup&gt;-1&lt;/sup&gt; were present in the samples, with loadings rising with time. Next generation Illumina MiSeq sequencing was performed to identify the dominant microorganisms at eight sampling times. The 16S rRNA gene sequence analysis suggested that 70% and 91% from of the OTUs samples, from the FT and INP respectively, belonged to the phylum Proteobacteria, mainly from the alpha and beta subclasses. The remaining OTUs were assigned primarily to the phyla Acidobacteria, Bacteroidetes, and, Cyanobacteria. Overall the most abundant genera identified were &lt;i&gt;Hydrogenophaga&lt;/i&gt;, &lt;i&gt;Curvibacter&lt;/i&gt;, &lt;i&gt;Porphyrobacter&lt;/i&gt;, &lt;i&gt;Rhodoferax&lt;/i&gt;, &lt;i&gt;Polaromonas&lt;/i&gt;, &lt;i&gt;Sediminibacterium&lt;/i&gt;, &lt;i&gt;Roseococcus&lt;/i&gt;, and &lt;i&gt;Sphingomonas.&lt;/i&gt; The presence of organisms most closely related to &lt;i&gt;Hydrogenophaga&lt;/i&gt; species in the INP areas, suggests the metabolism of hydrogen as an energy source, most likely linked to hydrolysis of water caused by the stored fuel. Isolation of axenic cultures using a range of minimal and rich media was also attempted, but only relatively minor components (from the phylum Bacteroidetes) of the pond water communities were obtained, emphasizing the importance of DNA-based, not culture-dependent techniques, for assessing the microbiome of nuclear facilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>636</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Ruminococcaceae_ucg-005</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
+      <c r="D75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>657</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Shinella</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Wu, H., Yang, M., Tsui, T., Yin, Z. &amp; Yin, C. (2020). Comparative evaluation on the utilization of applied electrical potential in a conductive granule packed biotrickling filter for continuous abatement of xylene: Performance, limitation, and microbial community.. Journal of environmental management, 274, 111145.</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>This study investigates the use of electrically conductive granules as packing material in biotrickling filter (BTF) systems as to provide insights on the specific microbial abundance and functions during the treatment of xylene-containing waste gas. In addition, the effect of applied potential on attached biofilm on conductive granules during xylene degradation was briefly investigated. During stable operation period, the conductive granules packed BTF achieved reactor performance of no less than 80% with a maximum EC of 137.7 g/m&lt;sup&gt;3&lt;/sup&gt; h. Under applied potential of 1V, the BTF system showed deterioration of xylene removal by ranging from 21 to 76%, which also affected the distribution and relative abundance of the major microorganisms such as Xanthobacter, Acidovorax, Rhodococcus, Hydrogenophaga, Arthrobacter, Brevundimonas, Pseudoxanthomonas, Devosia, Shinella, Sphingobium, Dokdonella, Pseudomonas and Bosea. The acclimation of applied potential led to the enrichment of autotrophic bacteria and strains, which are correlated to improved nitrogen cycling. In general, applying electrical potential is feasible to shape the microbiological structure of biofilms to selectively adjust their biochemical functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>678</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Sphingosinicella</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>712</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Tepidimonas</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>725</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Thermus</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Qureshi, K., et al. (2022). In Vitro and In Silico Approaches for the Evaluation of Antimicrobial Activity, Time-Kill Kinetics, and Anti-Biofilm Potential of Thymoquinone (2-Methyl-5-propan-2-ylcyclohexa-2,5-diene-1,4-dione) against Selected Human Pathogens.. Antibiotics (Basel, Switzerland), 11(1).</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Thymoquinone (2-methyl-5-propan-2-ylcyclohexa-2,5-diene-1,4-dione; TQ), a principal bioactive phytoconstituent of &lt;i&gt;Nigella sativa&lt;/i&gt; essential oil, has been reported to have high antimicrobial potential. Thus, the current study evaluated TQ's antimicrobial potential against a range of selected human pathogens using in vitro assays, including time-kill kinetics and anti-biofilm activity. In silico molecular docking of TQ against several antimicrobial target proteins and a detailed intermolecular interaction analysis was performed, including binding energies and docking feasibility. Of the tested bacteria and fungi, &lt;i&gt;S. epidermidis&lt;/i&gt; ATCC 12228 and &lt;i&gt;Candida albicans&lt;/i&gt; ATCC 10231 were the most susceptible to TQ, with 50.3 ± 0.3 mm and 21.1 ± 0.1 mm zones of inhibition, respectively. Minimum inhibitory concentration (MIC) values of TQ are in the range of 12.5-50 µg/mL, while minimum biocidal concentration (MBC) values are in the range of 25-100 µg/mL against the tested organisms. Time-kill kinetics of TQ revealed that the killing time for the tested bacteria is in the range of 1-6 h with the MBC of TQ. Anti-biofilm activity results demonstrate that the minimum biofilm inhibitory concentration (MBIC) values of TQ are in the range of 25-50 µg/mL, while the minimum biofilm eradication concentration (MBEC) values are in the range of 25-100 µg/mL, for the tested bacteria. In silico molecular docking studies revealed four preferred antibacterial and antifungal target proteins for TQ: D-alanyl-D-alanine synthetase (Ddl) from &lt;i&gt;Thermus thermophilus&lt;/i&gt;, transcriptional regulator qacR from &lt;i&gt;Staphylococcus aureus&lt;/i&gt;, N-myristoyltransferase from &lt;i&gt;Candida albicans&lt;/i&gt;, and NADPH-dependent D-xylose reductase from &lt;i&gt;Candida tenuis.&lt;/i&gt; In contrast, the nitroreductase family protein from &lt;i&gt;Bacillus cereus&lt;/i&gt; and spore coat polysaccharide biosynthesis protein from &lt;i&gt;Bacillus subtilis&lt;/i&gt; and UDP-N-acetylglucosamine pyrophosphorylase from &lt;i&gt;Aspergillus fumigatus&lt;/i&gt; are the least preferred antibacterial and antifungal target proteins for TQ, respectively. Molecular dynamics (MD) simulations revealed that TQ could bind to all four target proteins, with Ddl and NADPH-dependent D-xylose reductase being the most efficient. Our findings corroborate TQ's high antimicrobial potential, suggesting it may be a promising drug candidate for multi-drug resistant (MDR) pathogens, notably Gram-positive bacteria and &lt;i&gt;Candida albicans.&lt;/i&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>864</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Veillonella</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Sekar, P., Rizvi, Z., Abdullah, N., Samsudin, A. &amp; Kheder, W. (2025). Oral microbiota interactions with titanium implants: A pilot in-vivo and in-vitro study on the impact of peri-implantitis.. PloS one, 20(7), e0321428.</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Dental implant therapy is a reliable approach for restoring missing teeth, offering functional and aesthetic benefits in suitable clinical cases. However, there is still a 1.9-11% implant failure rate globally. Oral microbiota plays a significant role in implant failure and peri-implant infections. Hence the impact of oral microbiota on titanium dental implants, particularly in the context of dysbiosis and peri-implant diseases, was investigated by in-vivo and in-vitro methods in this study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>871</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Xanthobacter</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Wu, H., Yang, M., Tsui, T., Yin, Z. &amp; Yin, C. (2020). Comparative evaluation on the utilization of applied electrical potential in a conductive granule packed biotrickling filter for continuous abatement of xylene: Performance, limitation, and microbial community.. Journal of environmental management, 274, 111145.</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>This study investigates the use of electrically conductive granules as packing material in biotrickling filter (BTF) systems as to provide insights on the specific microbial abundance and functions during the treatment of xylene-containing waste gas. In addition, the effect of applied potential on attached biofilm on conductive granules during xylene degradation was briefly investigated. During stable operation period, the conductive granules packed BTF achieved reactor performance of no less than 80% with a maximum EC of 137.7 g/m&lt;sup&gt;3&lt;/sup&gt; h. Under applied potential of 1V, the BTF system showed deterioration of xylene removal by ranging from 21 to 76%, which also affected the distribution and relative abundance of the major microorganisms such as Xanthobacter, Acidovorax, Rhodococcus, Hydrogenophaga, Arthrobacter, Brevundimonas, Pseudoxanthomonas, Devosia, Shinella, Sphingobium, Dokdonella, Pseudomonas and Bosea. The acclimation of applied potential led to the enrichment of autotrophic bacteria and strains, which are correlated to improved nitrogen cycling. In general, applying electrical potential is feasible to shape the microbiological structure of biofilms to selectively adjust their biochemical functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>872</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Xanthomonadaceae_bacterium_wwh73</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Chung, K., Fujiki, I. &amp; Okabe, S. (2011). Effect of formation of biofilms and chemical scale on the cathode electrode on the performance of a continuous two-chamber microbial fuel cell.. Bioresource technology, 102(1), 355-60.</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>A two-chamber MFC system was operated continuously for more than 500 days to evaluate effects of biofilm and chemical scale formation on the cathode electrode on power generation. A stable power density of 0.57 W/m(2) was attained after 200 days operation. However, the power density decreased drastically to 0.2 W/m(2) after the cathodic biofilm and chemical scale were removed. As the cathodic biofilm and chemical scale partially accumulated on the cathode, the power density gradually recovered with time. Microbial community structure of the cathodic biofilm was analyzed based on 16S rRNA clone libraries. The clones closely related to Xanthomonadaceae bacterium and Xanthomonas sp. in the Gammaproteobacteria subdivision were most frequently retrieved from the cathodic biofilm. Results of the SEM-EDX analysis revealed that the cation species (Na(+) and Ca(2+)) were main constituents of chemical scale, indicating that these cations diffused from the anode chamber through the Nafion membrane. However, an excess accumulation of the biofilm and chemical scale on the cathode exhibited adverse effects on the power generation due to a decrease in the active cathode surface area and an increase in diffusion resistance for oxygen. Thus, it is important to properly control the formation of chemical scale and biofilm on the cathode during long-term operation.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>